<commit_message>
SAMA BCM: restructure per maintainer review (#4385)
- Render each subdomain Principle and Objective as Markdown headers in the
  description field.
- Split the lettered sub-points (a/b/c) of each control consideration into
  separate assessable child requirements.
- A consideration that only introduces a list (text ends with a colon) is now a
  non-assessable header; standalone considerations remain assessable.
- Make the library and framework descriptions identical and add the source link.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/excel/sama_bcm/sama-bcm-1.0.xlsx
+++ b/tools/excel/sama_bcm/sama-bcm-1.0.xlsx
@@ -448,7 +448,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SAMA Business Continuity Management (BCM) Framework, issued by the Saudi Central Bank (SAMA) for its Member Organizations (banks, insurance and finance companies, and payment service providers). The framework defines the BCM domains, subdomains, principles, objectives and control considerations for building organizational resilience, and is aligned with ISO 22301. 13 subdomains / 75 control considerations. Reference: https://rulebook.sama.gov.sa</t>
+          <t>SAMA Business Continuity Management (BCM) Framework, issued by the Saudi Central Bank (SAMA) for its Member Organizations (banks, insurance and finance companies, and payment service providers). It defines the BCM domains, subdomains, principles, objectives and control considerations for building organizational resilience, and is aligned with ISO 22301. 1 domain / 13 subdomains / 75 control considerations. Source: https://rulebook.sama.gov.sa/en/business-continuity-management-framework-1</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SAMA Business Continuity Management (BCM) Framework. One domain, 13 subdomains, 75 control considerations. Aligned with ISO 22301.</t>
+          <t>SAMA Business Continuity Management (BCM) Framework, issued by the Saudi Central Bank (SAMA) for its Member Organizations (banks, insurance and finance companies, and payment service providers). It defines the BCM domains, subdomains, principles, objectives and control considerations for building organizational resilience, and is aligned with ISO 22301. 1 domain / 13 subdomains / 75 control considerations. Source: https://rulebook.sama.gov.sa/en/business-continuity-management-framework-1</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -743,7 +743,10 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>The business continuity governance framework should be defined, approved, implemented and maintained, which should be monitored by senior management. The business continuity structure should be defined and communicated to all relevant employees and third parties. To direct, control and evaluate the overall approach to business continuity within the Member Organization</t>
+          <t>## Principle
+The business continuity governance framework should be defined, approved, implemented and maintained, which should be monitored by senior management. The business continuity structure should be defined and communicated to all relevant employees and third parties.
+## Objective
+To direct, control and evaluate the overall approach to business continuity within the Member Organization</t>
         </is>
       </c>
     </row>
@@ -832,11 +835,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
         <v>3</v>
       </c>
@@ -848,7 +847,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A business continuity committee charter should be developed and should reflect: (a) Committee objectives (b) Roles and responsibilities (c) Minimum number of meeting participants (d) Meeting frequency (minimum on quarterly basis)</t>
+          <t>A business continuity committee charter should be developed and should reflect:</t>
         </is>
       </c>
     </row>
@@ -859,17 +858,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.1-6</t>
+          <t>2.1-5.a</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A BCM function should be established.</t>
+          <t>Committee objectives</t>
         </is>
       </c>
     </row>
@@ -880,17 +879,17 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.1-7</t>
+          <t>2.1-5.b</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A BCM manager/head should: (a) Be appointed (b) Have appropriate authority to manage the BCM program (c) Be qualified and have appropriate experience, skills and competencies to implement and maintain the BCM program within the member organization</t>
+          <t>Roles and responsibilities</t>
         </is>
       </c>
     </row>
@@ -901,17 +900,17 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2.1-8</t>
+          <t>2.1-5.c</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The BCM function should be adequately staffed with qualified team members</t>
+          <t>Minimum number of meeting participants</t>
         </is>
       </c>
     </row>
@@ -922,59 +921,55 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.1-9</t>
+          <t>2.1-5.d</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cross-functional teams, consisting of strategic, tactical and operations team members should contribute in implementation and maintenance of the business continuity and disaster recovery plans.</t>
+          <t>Meeting frequency (minimum on quarterly basis)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>BCM Strategy</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>A business continuity strategy should be defined and aligned with the Member Organization's overall strategic business objectives. To ensure that business continuity Initiatives are in alignment with the strategic business objectives and embeds BCM as part of the good management practice within the Member Organization, in order to continual improvement In maturity.</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2.1-6</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A BCM function should be established.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
         <v>3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.2-1</t>
+          <t>2.1-7</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The business continuity strategy should be defined, approved, implemented and maintained.</t>
+          <t>A BCM manager/head should:</t>
         </is>
       </c>
     </row>
@@ -985,38 +980,38 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.2-2</t>
+          <t>2.1-7.a</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>The strategy should at minimum define: (a) Long-term strategic objectives for implementing and maturing the BCM program (b) Road map with timelines for achieving strategic objectives (c) Requirements for continual review and validation of alignment of the BCM program with strategic objectives</t>
+          <t>Be appointed</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Business Continuity Policy</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>A business continuity policy should be defined, approved and communicated to relevant stakeholders. To document the Member Organization’s commitment and objective of the business continuity program, and to communicate this to the relevant stakeholders.</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2.1-7.b</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Have appropriate authority to manage the BCM program</t>
         </is>
       </c>
     </row>
@@ -1027,17 +1022,17 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.3-1</t>
+          <t>2.1-7.c</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A business continuity policy should be defined, approved, implemented and communicated</t>
+          <t>Be qualified and have appropriate experience, skills and competencies to implement and maintain the BCM program within the member organization</t>
         </is>
       </c>
     </row>
@@ -1052,13 +1047,13 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.3-2</t>
+          <t>2.1-8</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>The business continuity policy should at the minimum identify: (a) Objectives (b) Scope (c) Responsibilities</t>
+          <t>The BCM function should be adequately staffed with qualified team members</t>
         </is>
       </c>
     </row>
@@ -1073,34 +1068,37 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2.3-3</t>
+          <t>2.1-9</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The compliance with the business continuity policy should be monitored .</t>
+          <t>Cross-functional teams, consisting of strategic, tactical and operations team members should contribute in implementation and maintenance of the business continuity and disaster recovery plans.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>3</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2.3-4</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>The effectiveness of policy implementation should be measured and periodically evaluated.</t>
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>BCM Strategy</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+A business continuity strategy should be defined and aligned with the Member Organization's overall strategic business objectives.
+## Objective
+To ensure that business continuity Initiatives are in alignment with the strategic business objectives and embeds BCM as part of the good management practice within the Member Organization, in order to continual improvement In maturity.</t>
         </is>
       </c>
     </row>
@@ -1115,34 +1113,30 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2.3-5</t>
+          <t>2.2-1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Scope exclusions for the BCM should be documented and periodically evaluated. The justifications for scope exclusions should be documented and approved by BCM committee and senior management.</t>
+          <t>The business continuity strategy should be defined, approved, implemented and maintained.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Business Impact Analysis (BIA) and Risk Assessment (RA)</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should perform a business impact analysis and risk assessment for all relevant activities to determine the business continuity, and disaster recovery requirements and improvements. To ensure that each Member Organization has Identified and prioritized their business processes along with key dependencies, and identified adequate controls in order to fulfill their business, regulatory, legal and compliance requirements with regards to business continuity</t>
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2.2-2</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>The strategy should at minimum define:</t>
         </is>
       </c>
     </row>
@@ -1153,17 +1147,17 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.4-1</t>
+          <t>2.2-2.a</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Methodology for BIA and RA should be defined, approved, implemented and maintained.</t>
+          <t>Long-term strategic objectives for implementing and maturing the BCM program</t>
         </is>
       </c>
     </row>
@@ -1174,17 +1168,17 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2.4-2</t>
+          <t>2.2-2.b</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>The Member Organization should periodically perform a Business Continuity risk assessment. It should include, but not limited to: (a) Identify potential internal and external threats, Including single point of failures that may cause disruption to critical activities as determined in the BIA considering people, process, technology and premises (b) Assess and prioritize potential risks by evaluating potential threats based on their operational impact and probability of occurrence (c) Select required controls to manage identified risks (d) Define treatment plan and implement BCM controls</t>
+          <t>Road map with timelines for achieving strategic objectives</t>
         </is>
       </c>
     </row>
@@ -1195,38 +1189,41 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.4-3</t>
+          <t>2.2-2.c</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>The Member Organization should identify and prioritize the activities (Le., products, services, business functions and processes) by performing BIA to determine the following but no limited to: (a) The potential impact of business disruptions for each prioritized business function and processes, including but not restricted to financial, operational, customer, legal and regulatory impacts (b) The recovery time objectives (RTOs), recover/ point objectives (RPOs) and maximum Acceptable Outage (MAO) (c) The internal and external interdependencies (d) Supporting recovery resources</t>
+          <t>Requirements for continual review and validation of alignment of the BCM program with strategic objectives</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2.4-4</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>The BCM committee should endorse the prioritized list, BIA results, RA and the defined RTOs, RPOs and MAOs.</t>
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Business Continuity Policy</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+A business continuity policy should be defined, approved and communicated to relevant stakeholders.
+## Objective
+To document the Member Organization’s commitment and objective of the business continuity program, and to communicate this to the relevant stakeholders.</t>
         </is>
       </c>
     </row>
@@ -1241,34 +1238,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2.4-5</t>
+          <t>2.3-1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Risk assessment results should be communicated to the BCM committee</t>
+          <t>A business continuity policy should be defined, approved, implemented and communicated</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
         <v>3</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2.4-6</t>
+          <t>2.3-2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>The BIA and RA should be updated annually and when major changes occur (such as change in structure and organization of people, process, technology, suppliers and locations).</t>
+          <t>The business continuity policy should at the minimum identify:</t>
         </is>
       </c>
     </row>
@@ -1279,17 +1272,17 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2.4-7</t>
+          <t>2.3-2.a</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>The risk assessment should include risks associated with overall organization as well as data centers (primary and alternative), which are not owned by the Member Organization (e.g., consider the timeframe needed to relocate to a new site and accordingly, It should Include a sufficient timeframe in the contractual agreement)</t>
+          <t>Objectives</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1293,17 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2.4-8</t>
+          <t>2.3-2.b</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Capability of vendors, suppliers and service providers to support and maintain service levels for prioritized activities during disruptive incidents should be assessed at least on a yearly basis.</t>
+          <t>Scope</t>
         </is>
       </c>
     </row>
@@ -1321,38 +1314,38 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2.4-9</t>
+          <t>2.3-2.c</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Member Organizations should ensure that RTOs are adequately defined for payment systems, customer related services, etc. considering the high availability of these operations and minimum disruption in the event of disaster.</t>
+          <t>Responsibilities</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Business Continuity Plan (BCP)</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should define, approve and Implement BCP for their critical activities. The compliance with BCP should be monitored, and the effectiveness should be measured and periodically evaluated. To ensure that the Member Organization has the capability to identify and clearly define the actions to be taken, and resources which are needed to enable the organization in managing a disruptive interruption and to come back to a position where normal business processes can resume</t>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2.3-3</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>The compliance with the business continuity policy should be monitored .</t>
         </is>
       </c>
     </row>
@@ -1367,13 +1360,13 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2.5-1</t>
+          <t>2.3-4</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A BCP should be defined, approved, implemented and maintained in readiness for use during disruptive incidents, to enable the Member organization to continue delivering its important and urgent activities, at an acceptable pre-defined level.</t>
+          <t>The effectiveness of policy implementation should be measured and periodically evaluated.</t>
         </is>
       </c>
     </row>
@@ -1388,34 +1381,37 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2.5-2</t>
+          <t>2.3-5</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>The member organization should define, approve and implement procedures for responding to disruptive incidents. The procedures should collectively include: (a) Key resources (e.g., people, equipment, facilities, technologies) (b) Defined roles, responsibilities and authorities for stakeholders (c) A process to manage the immediate consequences of a disruptive incident and escalation procedures (d) A process to continue the critical activities within predetermined recovery objectives (RTO, RPO and MAO) (e) A process to resume the Member Organization's operations to business-as-usual once the incident is resolved (f) Guidelines for communicating with employees, relevant third-parties and emergency contacts (g) Process for including relevant cyber security requirements, if any, within the business continuity planning</t>
+          <t>Scope exclusions for the BCM should be documented and periodically evaluated. The justifications for scope exclusions should be documented and approved by BCM committee and senior management.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>3</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2.5-3</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>The compliance with the BCP should be monitored.</t>
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Business Impact Analysis (BIA) and Risk Assessment (RA)</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should perform a business impact analysis and risk assessment for all relevant activities to determine the business continuity, and disaster recovery requirements and improvements.
+## Objective
+To ensure that each Member Organization has Identified and prioritized their business processes along with key dependencies, and identified adequate controls in order to fulfill their business, regulatory, legal and compliance requirements with regards to business continuity</t>
         </is>
       </c>
     </row>
@@ -1430,34 +1426,30 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2.5-4</t>
+          <t>2.4-1</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>The effectiveness of the BCPs should be measured and periodically evaluated.</t>
+          <t>Methodology for BIA and RA should be defined, approved, implemented and maintained.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
         <v>3</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2.5-5</t>
+          <t>2.4-2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>The BCM Manager and BCM coordinators are responsible to maintain and keep the BCPs and arrangements up-to-date.</t>
+          <t>The Member Organization should periodically perform a Business Continuity risk assessment. It should include, but not limited to:</t>
         </is>
       </c>
     </row>
@@ -1468,17 +1460,17 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2.5-6</t>
+          <t>2.4-2.a</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>The Member Organization should have sufficient alternative business workspace(s) where it can relocate the required resources to deliver the critical processes required as per predefined recovery objectives in the BIA.</t>
+          <t>Identify potential internal and external threats, Including single point of failures that may cause disruption to critical activities as determined in the BIA considering people, process, technology and premises</t>
         </is>
       </c>
     </row>
@@ -1489,17 +1481,17 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2.5-7</t>
+          <t>2.4-2.b</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>The alternative business workspace(s) should have clear demarcation of the sitting arrangement for different business units.</t>
+          <t>Assess and prioritize potential risks by evaluating potential threats based on their operational impact and probability of occurrence</t>
         </is>
       </c>
     </row>
@@ -1510,17 +1502,17 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2.5-8</t>
+          <t>2.4-2.c</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>The Member Organization should implement sufficient logical, physical and environmental security controls in order to support the same level of access and security in case the alternative location needs to be activated.</t>
+          <t>Select required controls to manage identified risks</t>
         </is>
       </c>
     </row>
@@ -1531,38 +1523,34 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2.5-10</t>
+          <t>2.4-2.d</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>For all critical activities, as determined by the BIA, the Member Organization should ensure that the key service providers (if any) have a BCP in place and their plans tested at least on a yearly basis.</t>
+          <t>Define treatment plan and implement BCM controls</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr"/>
-      <c r="B42" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>IT Disaster Recovery Plan (DRP)</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should define, approve, implement and maintain a IT DRP for its critical activities and related technology infrastructure. To ensure the Member Organization has IT DRP and up-to-date list of critical activities in place, in case of a disruptive incident</t>
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2.4-3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>The Member Organization should identify and prioritize the activities (Le., products, services, business functions and processes) by performing BIA to determine the following but no limited to:</t>
         </is>
       </c>
     </row>
@@ -1573,17 +1561,17 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2.6-1</t>
+          <t>2.4-3.a</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>An IT DRP to recover and restore technology services and infrastructure components (Data, systems, network, services and applications) should be defined, approved, implemented and maintained in alignment with business impact analysis.</t>
+          <t>The potential impact of business disruptions for each prioritized business function and processes, including but not restricted to financial, operational, customer, legal and regulatory impacts</t>
         </is>
       </c>
     </row>
@@ -1594,17 +1582,17 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2.6-2</t>
+          <t>2.4-3.b</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>The Member Organization should establish an alternative data center at an appropriate location. The location should be identified based on: (a) A risk assessment to confirm that the location does not share the same risks of the main data center (e.g., geographical threat) (b) Upon approval from SAMA</t>
+          <t>The recovery time objectives (RTOs), recover/ point objectives (RPOs) and maximum Acceptable Outage (MAO)</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1603,17 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2.6-3</t>
+          <t>2.4-3.c</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Data, system, network and application configurations, and capacities in the alternative data center should be commensurate to such configurations and capacities maintained in the main data center.</t>
+          <t>The internal and external interdependencies</t>
         </is>
       </c>
     </row>
@@ -1636,17 +1624,17 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2.6-4</t>
+          <t>2.4-3.d</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Member Organization should implement the same logical, physical, environmental and cyber security controls for the alternative data center as for the primary data center.</t>
+          <t>Supporting recovery resources</t>
         </is>
       </c>
     </row>
@@ -1661,13 +1649,13 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2.6-5</t>
+          <t>2.4-4</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>The Member Organization should define and implement a backup and recovery process.</t>
+          <t>The BCM committee should endorse the prioritized list, BIA results, RA and the defined RTOs, RPOs and MAOs.</t>
         </is>
       </c>
     </row>
@@ -1682,13 +1670,13 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2.6-6</t>
+          <t>2.4-5</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>The Member Organization should have offsite location for storing backups.</t>
+          <t>Risk assessment results should be communicated to the BCM committee</t>
         </is>
       </c>
     </row>
@@ -1703,13 +1691,13 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2.6-7</t>
+          <t>2.4-6</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Formal contracts should be signed with third parties to ensure the continuity of outsourced services or delivery of replacing hardware or software within the agreed timelines in case of a disaster. Include guidelines to ensure that the contracts signed with external service providers are aligned with the BIA and RA outcomes.</t>
+          <t>The BIA and RA should be updated annually and when major changes occur (such as change in structure and organization of people, process, technology, suppliers and locations).</t>
         </is>
       </c>
     </row>
@@ -1724,13 +1712,13 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2.6-8</t>
+          <t>2.4-7</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>The IT manager should be responsible to maintain and keep the disaster recovery plans and arrangements up to date with an overall accountability of integration within the BCM Program on the BCM Manager.</t>
+          <t>The risk assessment should include risks associated with overall organization as well as data centers (primary and alternative), which are not owned by the Member Organization (e.g., consider the timeframe needed to relocate to a new site and accordingly, It should Include a sufficient timeframe in the contractual agreement)</t>
         </is>
       </c>
     </row>
@@ -1745,13 +1733,13 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2.6-9</t>
+          <t>2.4-8</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>The compliance with the disaster recovery plan should be monitored.</t>
+          <t>Capability of vendors, suppliers and service providers to support and maintain service levels for prioritized activities during disruptive incidents should be assessed at least on a yearly basis.</t>
         </is>
       </c>
     </row>
@@ -1766,13 +1754,13 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2.6-10</t>
+          <t>2.4-9</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>The effectiveness of the IT DRP should be measured and should be evaluated on a yearly basis as minimum.</t>
+          <t>Member Organizations should ensure that RTOs are adequately defined for payment systems, customer related services, etc. considering the high availability of these operations and minimum disruption in the event of disaster.</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1771,20 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Cyber Resilience</t>
+          <t>Business Continuity Plan (BCP)</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>The Member Organization should ensure that critical services, business functions and processes run on reliable and robust infrastructure and software. To ensure each that the Member Organization's critical services, business functions and processes are available when required and resistant to disruptions.</t>
+          <t>## Principle
+The Member Organization should define, approve and Implement BCP for their critical activities. The compliance with BCP should be monitored, and the effectiveness should be measured and periodically evaluated.
+## Objective
+To ensure that the Member Organization has the capability to identify and clearly define the actions to be taken, and resources which are needed to enable the organization in managing a disruptive interruption and to come back to a position where normal business processes can resume</t>
         </is>
       </c>
     </row>
@@ -1808,55 +1799,51 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2.7-1</t>
+          <t>2.5-1</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>All changes to the infrastructure and software, which directly support the identified critical services, business functions and processes, should: (a) Be subject to in-depth risk assessments to ensure the agreed business requirements regarding availability and recovery are met. (b) Follow strict development, testing and change management procedures to avoid single point of failures or malfunctioning.</t>
+          <t>A BCP should be defined, approved, implemented and maintained in readiness for use during disruptive incidents, to enable the Member organization to continue delivering its important and urgent activities, at an acceptable pre-defined level.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
         <v>3</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2.7-2</t>
+          <t>2.5-2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>A periodic architectural review should be defined and approved to ensure the business requirements regarding availability and business continuity are being correctly addressed and implemented. _Note. For more control considerations to improve the overall resilience, e.g.,_[_threat management_](https://rulebook.sama.gov.sa/en/node/3958)_,_[_vulnerability management_](https://rulebook.sama.gov.sa/en/node/3960)_, please refer to the SAMA -_[_Cyber Security Framework_](https://rulebook.sama.gov.sa/en/node/3837)_._</t>
+          <t>The member organization should define, approve and implement procedures for responding to disruptive incidents. The procedures should collectively include:</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr"/>
-      <c r="B56" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Crisis Management Plan</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should define, approve and implement a crisis management plan that would facilitate a well-managed response for major incidents, including rapid communication to ensure overall safety to both internal and external stakeholders. To ensure the Member Organization has effective crisis management plan in place and up-to-date for critical member organization products, services, business functions and processes, in case of a disruptive incident.</t>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2.5-2.a</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Key resources (e.g., people, equipment, facilities, technologies)</t>
         </is>
       </c>
     </row>
@@ -1867,17 +1854,17 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2.8-1</t>
+          <t>2.5-2.b</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>A crisis management plan should be defined, approved and implemented.</t>
+          <t>Defined roles, responsibilities and authorities for stakeholders</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1875,17 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2.8-2</t>
+          <t>2.5-2.c</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>The compliance with the crisis management plan should be monitored.</t>
+          <t>A process to manage the immediate consequences of a disruptive incident and escalation procedures</t>
         </is>
       </c>
     </row>
@@ -1909,17 +1896,17 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2.8-3</t>
+          <t>2.5-2.d</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>The effectiveness of the business continuity program within the crisis management plan should be measured and periodically evaluated.</t>
+          <t>A process to continue the critical activities within predetermined recovery objectives (RTO, RPO and MAO)</t>
         </is>
       </c>
     </row>
@@ -1930,57 +1917,61 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2.8-4</t>
+          <t>2.5-2.e</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>The Member Organization should document a crisis management plan(s) that define(s) how crisis resulting from a major incident(s) will be addressed and managed, and should include at least: (a) Criteria for declaring a crisis. (b) The member organization should establish a command center for centralized management and an emergency command center. (c) Crisis-management team members. Considering representatives of the critical products, services, functions and processes of the Member Organization (including Communications department) (d) Contact details of those who are part of the crisis management team (including third-parties) (e) Definition of the steps to be taken during and after a crisis or disaster (including the mandates required) (f) Communication plan including the media response plan, to address the communication with the internal and external stakeholders during crisis. (g) The frequency of crisis management tests</t>
+          <t>A process to resume the Member Organization's operations to business-as-usual once the incident is resolved</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="inlineStr"/>
-      <c r="B61" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>2.9</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Testing</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should define, approve, implement, execute and monitor regular BCP and DRP tests to train their employees and third-parties and test the effectiveness of the BC and DR plans. To ensure that the Member Organization's existing BCP and DRP do work as defined and employees and third- parties are trained to execute these plans.</t>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2.5-2.f</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Guidelines for communicating with employees, relevant third-parties and emergency contacts</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="inlineStr"/>
-      <c r="B62" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>2.9.1</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>BCP Testing</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="inlineStr"/>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2.5-2.g</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Process for including relevant cyber security requirements, if any, within the business continuity planning</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1989,17 +1980,17 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2.9.1-1</t>
+          <t>2.5-3</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>The Member Organization should periodically conduct BCP simulation test exercises ("at least once a year")</t>
+          <t>The compliance with the BCP should be monitored.</t>
         </is>
       </c>
     </row>
@@ -2010,17 +2001,17 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2.9.1-2</t>
+          <t>2.5-4</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>The tests should consider appropriate scenarios that are well planned with clearly defined objectives (e.g., per function, per service, per process, per location, per worst cases scenarios). The Member Organization should take into consideration to Include cyber security scenarios.</t>
+          <t>The effectiveness of the BCPs should be measured and periodically evaluated.</t>
         </is>
       </c>
     </row>
@@ -2031,17 +2022,17 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2.9.1-3</t>
+          <t>2.5-5</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Defined test scenarios should cover the activation and involvement for crisis management team.</t>
+          <t>The BCM Manager and BCM coordinators are responsible to maintain and keep the BCPs and arrangements up-to-date.</t>
         </is>
       </c>
     </row>
@@ -2052,36 +2043,40 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2.9.1-4</t>
+          <t>2.5-6</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>After the completion of the above individual tests, each Member organization should consider conducting an integrated BCM test for all critical services, business processes and functions.</t>
+          <t>The Member Organization should have sufficient alternative business workspace(s) where it can relocate the required resources to deliver the critical processes required as per predefined recovery objectives in the BIA.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr"/>
-      <c r="B67" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>2.9.2</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>DRP Testing</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr"/>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2.5-7</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>The alternative business workspace(s) should have clear demarcation of the sitting arrangement for different business units.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2090,17 +2085,17 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2.9.2-1</t>
+          <t>2.5-8</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>The Member Organization should periodically execute a DR test combined with BCP ("at least once a year").</t>
+          <t>The Member Organization should implement sufficient logical, physical and environmental security controls in order to support the same level of access and security in case the alternative location needs to be activated.</t>
         </is>
       </c>
     </row>
@@ -2111,38 +2106,41 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2.9.2-2</t>
+          <t>2.5-10</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>The Member Organization should conduct an evaluation of the executed DR test of IT DR infrastructure that supports the Member Organization's critical systems to ensure the readiness and capability of DR to resume critical business operations for a period of time in case of a major disaster.</t>
+          <t>For all critical activities, as determined by the BIA, the Member Organization should ensure that the key service providers (if any) have a BCP in place and their plans tested at least on a yearly basis.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>4</v>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>2.9.2-3</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>The DR test results should provide an evaluation and suggestions for improvements to manage disruptive events impacting the Member Organization's business continuity.</t>
+      <c r="A70" s="5" t="inlineStr"/>
+      <c r="B70" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>IT Disaster Recovery Plan (DRP)</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should define, approve, implement and maintain a IT DRP for its critical activities and related technology infrastructure.
+## Objective
+To ensure the Member Organization has IT DRP and up-to-date list of critical activities in place, in case of a disruptive incident</t>
         </is>
       </c>
     </row>
@@ -2153,36 +2151,36 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2.9.2-4</t>
+          <t>2.6-1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>It should cover the activation and involvement of the crisis management team.</t>
+          <t>An IT DRP to recover and restore technology services and infrastructure components (Data, systems, network, services and applications) should be defined, approved, implemented and maintained in alignment with business impact analysis.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="inlineStr"/>
-      <c r="B72" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>2.9.3</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Executed Tests</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr"/>
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2.6-2</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>The Member Organization should establish an alternative data center at an appropriate location. The location should be identified based on:</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2195,13 +2193,13 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2.9.3-1</t>
+          <t>2.6-2.a</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Detailed results of all exercises and tests should be documented for future reference. The exercises/tests results should include, but not be limited to the following considerations: (a) Confirm meeting the objectives of the exercised plan (b) Confirm capabilities and readiness of recovery resources (c) Document lessons learnt and the required improvements (d) In case of failure, Capture the root-cause of the failure and remediation actions should be tracked to successful conclusion</t>
+          <t>A risk assessment to confirm that the location does not share the same risks of the main data center (e.g., geographical threat)</t>
         </is>
       </c>
     </row>
@@ -2216,13 +2214,13 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2.9.3-2</t>
+          <t>2.6-2.b</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Re-testing of the plan within the defined timelines in case of a failure, the timelines should not exceed the limit of three (3) months.</t>
+          <t>Upon approval from SAMA</t>
         </is>
       </c>
     </row>
@@ -2233,17 +2231,17 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2.9.3-3</t>
+          <t>2.6-3</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>The Internal Audit of the Member Organization, or a qualified external auditor, should observe the business continuity and disaster recovery testing activities as an independent participant in order to provide a reasonable assurance on the executed activities, test results and to observe if the executed tests are meeting the Member Organization's overall Business Continuity program objectives.</t>
+          <t>Data, system, network and application configurations, and capacities in the alternative data center should be commensurate to such configurations and capacities maintained in the main data center.</t>
         </is>
       </c>
     </row>
@@ -2254,38 +2252,38 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2.9.3-4</t>
+          <t>2.6-4</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>All BCP and DRP tests results should be reported to the BCM committee, senior management and the board of directors.</t>
+          <t>Member Organization should implement the same logical, physical, environmental and cyber security controls for the alternative data center as for the primary data center.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="inlineStr"/>
-      <c r="B77" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>Awareness and Training</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should establish, Implement and maintain a training and awareness program that effectively supports the BCM objectives by developing the required competency among staff. The Member Organization should ensure BCM integration into its day-to-day activities, through an ongoing awareness plan, which should be documented.</t>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2.6-5</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>The Member Organization should define and implement a backup and recovery process.</t>
         </is>
       </c>
     </row>
@@ -2300,13 +2298,13 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2.10-1</t>
+          <t>2.6-6</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>The Member Organization and relevant third-parties, such as providers and suppliers should be: (a) Familiar with relevant parts of business continuity policy and plans (b) Contractually bound to provide their services or products within the agreed time, in case of disruptive event (c) Familiar with their point of contact or their local BCM coordinator in the Member Organization (d) Familiar with their roles and responsibilities during disruptive incidents</t>
+          <t>The Member Organization should have offsite location for storing backups.</t>
         </is>
       </c>
     </row>
@@ -2321,13 +2319,13 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2.10-2</t>
+          <t>2.6-7</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>A training program should be provided once on an annual basis to employees involved in BCM to achieve the required level of experience, skills and competences.</t>
+          <t>Formal contracts should be signed with third parties to ensure the continuity of outsourced services or delivery of replacing hardware or software within the agreed timelines in case of a disaster. Include guidelines to ensure that the contracts signed with external service providers are aligned with the BIA and RA outcomes.</t>
         </is>
       </c>
     </row>
@@ -2342,34 +2340,34 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2.10-3</t>
+          <t>2.6-8</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>The Member Organization should periodically measure the effectiveness of the training and awareness program.</t>
+          <t>The IT manager should be responsible to maintain and keep the disaster recovery plans and arrangements up to date with an overall accountability of integration within the BCM Program on the BCM Manager.</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="inlineStr"/>
-      <c r="B81" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>2.11</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>The Member Organization should define, establish and maintain a communication process for periodic communications with SAMA on matters related to its BCM program. To ensure that continuous communication is maintained with SAMA by defining, agreeing and adhering to communication protocol, frequency, and roles and responsibilities for communications</t>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>3</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2.6-9</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>The compliance with the disaster recovery plan should be monitored.</t>
         </is>
       </c>
     </row>
@@ -2384,55 +2382,54 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2.11-1</t>
+          <t>2.6-10</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
-          <t>The Member Organization should report all disruptive incidents classified as "Medium" or "High" to SAMA "Banking IT Risk Supervision" immediately. A post-incident report should be communicated to SAMA after the Member Organization resumes to normal operations.</t>
+          <t>The effectiveness of the IT DRP should be measured and should be evaluated on a yearly basis as minimum.</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>3</v>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>2.11-2</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>The Member Organization should coordinate with SAMA Supervision when communicating with the media in case of incidents.</t>
+      <c r="A83" s="5" t="inlineStr"/>
+      <c r="B83" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Cyber Resilience</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should ensure that critical services, business functions and processes run on reliable and robust infrastructure and software.
+## Objective
+To ensure each that the Member Organization's critical services, business functions and processes are available when required and resistant to disruptions.</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A84" t="inlineStr"/>
       <c r="B84" t="n">
         <v>3</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2.11-3</t>
+          <t>2.7-1</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Member Organizations should seek SAMA's approval when selecting a new site for its main or alternative data center, or when relocating the current main or alternative data center.</t>
+          <t>All changes to the infrastructure and software, which directly support the identified critical services, business functions and processes, should:</t>
         </is>
       </c>
     </row>
@@ -2443,17 +2440,17 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2.11-4</t>
+          <t>2.7-1.a</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>The Member Organization should communicate the approved program for executing business continuity and disaster recovery tests, for the upcoming year, with SAMA "Banking IT Risk Supervision" by end of January of every year.</t>
+          <t>Be subject to in-depth risk assessments to ensure the agreed business requirements regarding availability and recovery are met.</t>
         </is>
       </c>
     </row>
@@ -2464,59 +2461,62 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2.11-5</t>
+          <t>2.7-1.b</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Test results of business continuity and disaster recovery should be shared with SAMA within four weeks after the test The Member Organization should identify the improvements based on the test performed and provide an action plan to SAMA within two months after the submission of the test results.</t>
+          <t>Follow strict development, testing and change management procedures to avoid single point of failures or malfunctioning.</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="inlineStr"/>
-      <c r="B87" s="5" t="n">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>3</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2.7-2</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>A periodic architectural review should be defined and approved to ensure the business requirements regarding availability and business continuity are being correctly addressed and implemented. _Note. For more control considerations to improve the overall resilience, e.g.,_[_threat management_](https://rulebook.sama.gov.sa/en/node/3958)_,_[_vulnerability management_](https://rulebook.sama.gov.sa/en/node/3960)_, please refer to the SAMA -_[_Cyber Security Framework_](https://rulebook.sama.gov.sa/en/node/3837)_._</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr"/>
+      <c r="B88" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>2.12</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>Periodic Documents Review</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>The business continuity and disaster recovery program, policies, plans and procedures should be reviewed and updated periodically, and in case of (major) change in the Member Organization's critical products, services, business functions and/or processes. To ensure that all the business continuity documents are up to date and can be used during a disruptive incident to recover the business operations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>3</v>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>2.12-1</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Member Organizations should establish a process for document review/update to ensure the BC documents are up-to-date, reviewed and approved.</t>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Crisis Management Plan</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should define, approve and implement a crisis management plan that would facilitate a well-managed response for major incidents, including rapid communication to ensure overall safety to both internal and external stakeholders.
+## Objective
+To ensure the Member Organization has effective crisis management plan in place and up-to-date for critical member organization products, services, business functions and processes, in case of a disruptive incident.</t>
         </is>
       </c>
     </row>
@@ -2531,34 +2531,34 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2.12-2</t>
+          <t>2.8-1</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>All documents should clearly identify the last date in which the document was reviewed and approved.</t>
+          <t>A crisis management plan should be defined, approved and implemented.</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="inlineStr"/>
-      <c r="B90" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>Assurance</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>The BCM of the Member Organizations should be subjected to periodically reviews and audits by a qualified independent internal or external party to ensure its effectiveness, and to obtain assurance regarding the compliance with the SAMA BCM. To ensure that an independent party is reviewing the BCM framework activities and reporting the identified issues to the senior management independently.</t>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2.8-2</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>The compliance with the crisis management plan should be monitored.</t>
         </is>
       </c>
     </row>
@@ -2573,34 +2573,30 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2.13-1</t>
+          <t>2.8-3</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Member organization should conduct review / audit of BCM by qualified independent internal/ external party.</t>
+          <t>The effectiveness of the business continuity program within the crisis management plan should be measured and periodically evaluated.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
         <v>3</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2.13-2</t>
+          <t>2.8-4</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
-          <t>the Member Organization should identify the gaps and provide a road map to enhance the BCM within the organization.</t>
+          <t>The Member Organization should document a crisis management plan(s) that define(s) how crisis resulting from a major incident(s) will be addressed and managed, and should include at least:</t>
         </is>
       </c>
     </row>
@@ -2611,15 +2607,997 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2.13-3</t>
+          <t>2.8-4.a</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
+        <is>
+          <t>Criteria for declaring a crisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>4</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2.8-4.b</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>The member organization should establish a command center for centralized management and an emergency command center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>4</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2.8-4.c</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Crisis-management team members. Considering representatives of the critical products, services, functions and processes of the Member Organization (including Communications department)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>4</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2.8-4.d</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Contact details of those who are part of the crisis management team (including third-parties)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>4</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2.8-4.e</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Definition of the steps to be taken during and after a crisis or disaster (including the mandates required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>4</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2.8-4.f</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Communication plan including the media response plan, to address the communication with the internal and external stakeholders during crisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2.8-4.g</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>The frequency of crisis management tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr"/>
+      <c r="B100" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should define, approve, implement, execute and monitor regular BCP and DRP tests to train their employees and third-parties and test the effectiveness of the BC and DR plans.
+## Objective
+To ensure that the Member Organization's existing BCP and DRP do work as defined and employees and third- parties are trained to execute these plans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr"/>
+      <c r="B101" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>2.9.1</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>BCP Testing</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>4</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2.9.1-1</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>The Member Organization should periodically conduct BCP simulation test exercises ("at least once a year")</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>4</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2.9.1-2</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>The tests should consider appropriate scenarios that are well planned with clearly defined objectives (e.g., per function, per service, per process, per location, per worst cases scenarios). The Member Organization should take into consideration to Include cyber security scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>4</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2.9.1-3</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Defined test scenarios should cover the activation and involvement for crisis management team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2.9.1-4</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>After the completion of the above individual tests, each Member organization should consider conducting an integrated BCM test for all critical services, business processes and functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr"/>
+      <c r="B106" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>2.9.2</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>DRP Testing</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>4</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2.9.2-1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>The Member Organization should periodically execute a DR test combined with BCP ("at least once a year").</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>4</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2.9.2-2</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>The Member Organization should conduct an evaluation of the executed DR test of IT DR infrastructure that supports the Member Organization's critical systems to ensure the readiness and capability of DR to resume critical business operations for a period of time in case of a major disaster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>4</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2.9.2-3</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>The DR test results should provide an evaluation and suggestions for improvements to manage disruptive events impacting the Member Organization's business continuity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2.9.2-4</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>It should cover the activation and involvement of the crisis management team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr"/>
+      <c r="B111" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>2.9.3</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Executed Tests</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr"/>
+      <c r="B112" t="n">
+        <v>4</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2.9.3-1</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Detailed results of all exercises and tests should be documented for future reference. The exercises/tests results should include, but not be limited to the following considerations:</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>5</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2.9.3-1.a</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Confirm meeting the objectives of the exercised plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>5</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2.9.3-1.b</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Confirm capabilities and readiness of recovery resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>5</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2.9.3-1.c</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Document lessons learnt and the required improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>5</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2.9.3-1.d</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>In case of failure, Capture the root-cause of the failure and remediation actions should be tracked to successful conclusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>4</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2.9.3-2</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Re-testing of the plan within the defined timelines in case of a failure, the timelines should not exceed the limit of three (3) months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>4</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2.9.3-3</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>The Internal Audit of the Member Organization, or a qualified external auditor, should observe the business continuity and disaster recovery testing activities as an independent participant in order to provide a reasonable assurance on the executed activities, test results and to observe if the executed tests are meeting the Member Organization's overall Business Continuity program objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>4</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>2.9.3-4</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>All BCP and DRP tests results should be reported to the BCM committee, senior management and the board of directors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr"/>
+      <c r="B120" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>Awareness and Training</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should establish, Implement and maintain a training and awareness program that effectively supports the BCM objectives by developing the required competency among staff.
+## Objective
+The Member Organization should ensure BCM integration into its day-to-day activities, through an ongoing awareness plan, which should be documented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="n">
+        <v>3</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>2.10-1</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>The Member Organization and relevant third-parties, such as providers and suppliers should be:</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>4</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>2.10-1.a</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Familiar with relevant parts of business continuity policy and plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>4</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>2.10-1.b</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Contractually bound to provide their services or products within the agreed time, in case of disruptive event</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>4</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>2.10-1.c</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Familiar with their point of contact or their local BCM coordinator in the Member Organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>2.10-1.d</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Familiar with their roles and responsibilities during disruptive incidents</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>2.10-2</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>A training program should be provided once on an annual basis to employees involved in BCM to achieve the required level of experience, skills and competences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>3</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>2.10-3</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>The Member Organization should periodically measure the effectiveness of the training and awareness program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr"/>
+      <c r="B128" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The Member Organization should define, establish and maintain a communication process for periodic communications with SAMA on matters related to its BCM program.
+## Objective
+To ensure that continuous communication is maintained with SAMA by defining, agreeing and adhering to communication protocol, frequency, and roles and responsibilities for communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>3</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>2.11-1</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>The Member Organization should report all disruptive incidents classified as "Medium" or "High" to SAMA "Banking IT Risk Supervision" immediately. A post-incident report should be communicated to SAMA after the Member Organization resumes to normal operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>2.11-2</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>The Member Organization should coordinate with SAMA Supervision when communicating with the media in case of incidents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>3</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2.11-3</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Member Organizations should seek SAMA's approval when selecting a new site for its main or alternative data center, or when relocating the current main or alternative data center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>3</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2.11-4</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>The Member Organization should communicate the approved program for executing business continuity and disaster recovery tests, for the upcoming year, with SAMA "Banking IT Risk Supervision" by end of January of every year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>3</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2.11-5</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Test results of business continuity and disaster recovery should be shared with SAMA within four weeks after the test The Member Organization should identify the improvements based on the test performed and provide an action plan to SAMA within two months after the submission of the test results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr"/>
+      <c r="B134" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>Periodic Documents Review</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The business continuity and disaster recovery program, policies, plans and procedures should be reviewed and updated periodically, and in case of (major) change in the Member Organization's critical products, services, business functions and/or processes.
+## Objective
+To ensure that all the business continuity documents are up to date and can be used during a disruptive incident to recover the business operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>3</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>2.12-1</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Member Organizations should establish a process for document review/update to ensure the BC documents are up-to-date, reviewed and approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>3</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>2.12-2</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>All documents should clearly identify the last date in which the document was reviewed and approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr"/>
+      <c r="B137" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>Assurance</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>## Principle
+The BCM of the Member Organizations should be subjected to periodically reviews and audits by a qualified independent internal or external party to ensure its effectiveness, and to obtain assurance regarding the compliance with the SAMA BCM.
+## Objective
+To ensure that an independent party is reviewing the BCM framework activities and reporting the identified issues to the senior management independently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>3</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>2.13-1</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Member organization should conduct review / audit of BCM by qualified independent internal/ external party.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>3</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>2.13-2</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>the Member Organization should identify the gaps and provide a road map to enhance the BCM within the organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>3</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>2.13-3</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr">
         <is>
           <t>The identified gaps along with road map should be reported to senior management and BCM committee.</t>
         </is>

</xml_diff>